<commit_message>
Fix DataSample 20 Tables, Delete Unused Tables
</commit_message>
<xml_diff>
--- a/src/mocks/greenlight_data.xlsx
+++ b/src/mocks/greenlight_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SmartDrivingLearningSystem\smart_driving_learning_system\src\mocks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BFCAE98-A135-42CD-BCD9-664C9E4D9D47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09311508-7DE5-4B21-9F11-D23B9CC2813F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="14" activeTab="19" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Role" sheetId="1" r:id="rId1"/>
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10183" uniqueCount="2986">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10949" uniqueCount="3039">
   <si>
     <t>id</t>
   </si>
@@ -8963,42 +8963,12 @@
     <t>#28a745</t>
   </si>
   <si>
-    <t>lesson_1</t>
-  </si>
-  <si>
-    <t>description_lesson_1</t>
-  </si>
-  <si>
-    <t>lesson_2</t>
-  </si>
-  <si>
-    <t>description_lesson_2</t>
-  </si>
-  <si>
-    <t>chapter_1</t>
-  </si>
-  <si>
-    <t>description_chapter_1</t>
-  </si>
-  <si>
-    <t>chapter_2</t>
-  </si>
-  <si>
-    <t>description_chapter_2</t>
-  </si>
-  <si>
     <t>A1</t>
   </si>
   <si>
     <t>A2</t>
   </si>
   <si>
-    <t>content_1</t>
-  </si>
-  <si>
-    <t>content_2</t>
-  </si>
-  <si>
     <t>totakDuration</t>
   </si>
   <si>
@@ -9021,6 +8991,195 @@
   </si>
   <si>
     <t>simulationSessionId</t>
+  </si>
+  <si>
+    <t>123456a</t>
+  </si>
+  <si>
+    <t>Description of A1</t>
+  </si>
+  <si>
+    <t>Description of A2</t>
+  </si>
+  <si>
+    <t>Description of A3</t>
+  </si>
+  <si>
+    <t>Description of A4</t>
+  </si>
+  <si>
+    <t>Description of A5</t>
+  </si>
+  <si>
+    <t>Description of A6</t>
+  </si>
+  <si>
+    <t>A3</t>
+  </si>
+  <si>
+    <t>A4</t>
+  </si>
+  <si>
+    <t>A5</t>
+  </si>
+  <si>
+    <t>A6</t>
+  </si>
+  <si>
+    <t>Chapter 1</t>
+  </si>
+  <si>
+    <t>Chapter 2</t>
+  </si>
+  <si>
+    <t>Chapter 3</t>
+  </si>
+  <si>
+    <t>Chapter 4</t>
+  </si>
+  <si>
+    <t>Chapter 5</t>
+  </si>
+  <si>
+    <t>Chapter 6</t>
+  </si>
+  <si>
+    <t>Chapter 7</t>
+  </si>
+  <si>
+    <t>Chapter 8</t>
+  </si>
+  <si>
+    <t>Chapter 9</t>
+  </si>
+  <si>
+    <t>Chapter 10</t>
+  </si>
+  <si>
+    <t>Chapter 11</t>
+  </si>
+  <si>
+    <t>Chapter 12</t>
+  </si>
+  <si>
+    <t>Chapter 13</t>
+  </si>
+  <si>
+    <t>Chapter 14</t>
+  </si>
+  <si>
+    <t>Chapter 15</t>
+  </si>
+  <si>
+    <t>Description of Chapter 1</t>
+  </si>
+  <si>
+    <t>Description of Chapter 2</t>
+  </si>
+  <si>
+    <t>Description of Chapter 3</t>
+  </si>
+  <si>
+    <t>Description of Chapter 4</t>
+  </si>
+  <si>
+    <t>Description of Chapter 5</t>
+  </si>
+  <si>
+    <t>Lesson 1</t>
+  </si>
+  <si>
+    <t>Lesson 2</t>
+  </si>
+  <si>
+    <t>Lesson 3</t>
+  </si>
+  <si>
+    <t>Lesson 4</t>
+  </si>
+  <si>
+    <t>Lesson 5</t>
+  </si>
+  <si>
+    <t>Lesson 6</t>
+  </si>
+  <si>
+    <t>Lesson 7</t>
+  </si>
+  <si>
+    <t>Lesson 8</t>
+  </si>
+  <si>
+    <t>Lesson 9</t>
+  </si>
+  <si>
+    <t>Lesson 10</t>
+  </si>
+  <si>
+    <t>Description of Lesson 1</t>
+  </si>
+  <si>
+    <t>Description of Lesson 2</t>
+  </si>
+  <si>
+    <t>Description of Lesson 3</t>
+  </si>
+  <si>
+    <t>Description of Lesson 4</t>
+  </si>
+  <si>
+    <t>Description of Lesson 5</t>
+  </si>
+  <si>
+    <t>Description of Lesson 6</t>
+  </si>
+  <si>
+    <t>Description of Lesson 7</t>
+  </si>
+  <si>
+    <t>Description of Lesson 8</t>
+  </si>
+  <si>
+    <t>Description of Lesson 9</t>
+  </si>
+  <si>
+    <t>Description of Lesson 10</t>
+  </si>
+  <si>
+    <t>&lt;h2&gt;Bài học 1&lt;/h2&gt;&lt;p&gt;Nội dung bài học 1.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>&lt;h2&gt;Bài học 2&lt;/h2&gt;&lt;p&gt;Nội dung bài học 2.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>&lt;h2&gt;Bài học 3&lt;/h2&gt;&lt;p&gt;Nội dung bài học 3.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>&lt;h2&gt;Bài học 4&lt;/h2&gt;&lt;p&gt;Nội dung bài học 4.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>&lt;h2&gt;Bài học 5&lt;/h2&gt;&lt;p&gt;Nội dung bài học 5.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>&lt;h2&gt;Bài học 6&lt;/h2&gt;&lt;p&gt;Nội dung bài học 6.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>&lt;h2&gt;Bài học 7&lt;/h2&gt;&lt;p&gt;Nội dung bài học 7.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>&lt;h2&gt;Bài học 8&lt;/h2&gt;&lt;p&gt;Nội dung bài học 8.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>&lt;h2&gt;Bài học 9&lt;/h2&gt;&lt;p&gt;Nội dung bài học 9.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>&lt;h2&gt;Bài học 10&lt;/h2&gt;&lt;p&gt;Nội dung bài học 10.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>category_3</t>
+  </si>
+  <si>
+    <t>description_category_3</t>
   </si>
 </sst>
 </file>
@@ -9507,16 +9666,16 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>2981</v>
+        <v>2971</v>
       </c>
       <c r="C1" t="s">
         <v>16</v>
       </c>
       <c r="D1" t="s">
-        <v>2982</v>
+        <v>2972</v>
       </c>
       <c r="E1" t="s">
-        <v>2983</v>
+        <v>2973</v>
       </c>
       <c r="F1" t="s">
         <v>39</v>
@@ -9613,10 +9772,10 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>2984</v>
+        <v>2974</v>
       </c>
       <c r="C1" t="s">
-        <v>2985</v>
+        <v>2975</v>
       </c>
       <c r="D1" t="s">
         <v>37</v>
@@ -9693,12 +9852,12 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="17.28515625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="6.28515625" bestFit="1" customWidth="1"/>
   </cols>
@@ -9728,10 +9887,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>2974</v>
+        <v>2966</v>
       </c>
       <c r="C2" t="s">
-        <v>2919</v>
+        <v>2977</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>2946</v>
@@ -9748,10 +9907,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>2975</v>
+        <v>2967</v>
       </c>
       <c r="C3" t="s">
-        <v>2920</v>
+        <v>2978</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>2946</v>
@@ -9760,7 +9919,87 @@
         <v>2947</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>2983</v>
+      </c>
+      <c r="C4" t="s">
+        <v>2979</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="F4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>2984</v>
+      </c>
+      <c r="C5" t="s">
+        <v>2980</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="F5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>2985</v>
+      </c>
+      <c r="C6" t="s">
+        <v>2981</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="F6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>2986</v>
+      </c>
+      <c r="C7" t="s">
+        <v>2982</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="F7">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -9935,13 +10174,13 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="2.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="6" width="17.28515625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="6.28515625" bestFit="1" customWidth="1"/>
   </cols>
@@ -9977,10 +10216,10 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>2970</v>
+        <v>2987</v>
       </c>
       <c r="D2" t="s">
-        <v>2971</v>
+        <v>3002</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>2946</v>
@@ -9997,40 +10236,340 @@
         <v>2</v>
       </c>
       <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>2988</v>
+      </c>
+      <c r="D3" t="s">
+        <v>3003</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="G3">
         <v>2</v>
       </c>
-      <c r="C3" t="s">
-        <v>2972</v>
-      </c>
-      <c r="D3" t="s">
-        <v>2973</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>2946</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>2947</v>
-      </c>
-      <c r="G3">
-        <v>1</v>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4" t="s">
+        <v>2989</v>
+      </c>
+      <c r="D4" t="s">
+        <v>3004</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="G4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5" t="s">
+        <v>2990</v>
+      </c>
+      <c r="D5" t="s">
+        <v>3005</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="G5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6" t="s">
+        <v>2991</v>
+      </c>
+      <c r="D6" t="s">
+        <v>3006</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="G6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>2992</v>
+      </c>
+      <c r="D7" t="s">
+        <v>3002</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="G7">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>2</v>
+      </c>
+      <c r="C8" t="s">
+        <v>2993</v>
+      </c>
+      <c r="D8" t="s">
+        <v>3003</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="G8">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>2</v>
+      </c>
+      <c r="C9" t="s">
+        <v>2994</v>
+      </c>
+      <c r="D9" t="s">
+        <v>3004</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="G9">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>2</v>
+      </c>
+      <c r="C10" t="s">
+        <v>2995</v>
+      </c>
+      <c r="D10" t="s">
+        <v>3005</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="G10">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>3</v>
+      </c>
+      <c r="C11" t="s">
+        <v>2996</v>
+      </c>
+      <c r="D11" t="s">
+        <v>3002</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="G11">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12">
+        <v>3</v>
+      </c>
+      <c r="C12" t="s">
+        <v>2997</v>
+      </c>
+      <c r="D12" t="s">
+        <v>3003</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="G12">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>2998</v>
+      </c>
+      <c r="D13" t="s">
+        <v>3004</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="G13">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14">
+        <v>4</v>
+      </c>
+      <c r="C14" t="s">
+        <v>2999</v>
+      </c>
+      <c r="D14" t="s">
+        <v>3002</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="G14">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15">
+        <v>4</v>
+      </c>
+      <c r="C15" t="s">
+        <v>3000</v>
+      </c>
+      <c r="D15" t="s">
+        <v>3003</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="G15">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16">
+        <v>5</v>
+      </c>
+      <c r="C16" t="s">
+        <v>3001</v>
+      </c>
+      <c r="D16" t="s">
+        <v>3002</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="G16">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H141"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="2.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="44.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="17.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="6.28515625" bestFit="1" customWidth="1"/>
   </cols>
@@ -10069,13 +10608,13 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>2966</v>
+        <v>3007</v>
       </c>
       <c r="D2" t="s">
-        <v>2967</v>
+        <v>3017</v>
       </c>
       <c r="E2" t="s">
-        <v>2976</v>
+        <v>3027</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>2946</v>
@@ -10092,25 +10631,3613 @@
         <v>2</v>
       </c>
       <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>3008</v>
+      </c>
+      <c r="D3" t="s">
+        <v>3018</v>
+      </c>
+      <c r="E3" t="s">
+        <v>3028</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H3">
         <v>2</v>
       </c>
-      <c r="C3" t="s">
-        <v>2968</v>
-      </c>
-      <c r="D3" t="s">
-        <v>2969</v>
-      </c>
-      <c r="E3" t="s">
-        <v>2977</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>2946</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>2947</v>
-      </c>
-      <c r="H3">
-        <v>1</v>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4" t="s">
+        <v>3009</v>
+      </c>
+      <c r="D4" t="s">
+        <v>3019</v>
+      </c>
+      <c r="E4" t="s">
+        <v>3029</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5" t="s">
+        <v>3010</v>
+      </c>
+      <c r="D5" t="s">
+        <v>3020</v>
+      </c>
+      <c r="E5" t="s">
+        <v>3030</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6" t="s">
+        <v>3011</v>
+      </c>
+      <c r="D6" t="s">
+        <v>3021</v>
+      </c>
+      <c r="E6" t="s">
+        <v>3031</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7" t="s">
+        <v>3012</v>
+      </c>
+      <c r="D7" t="s">
+        <v>3022</v>
+      </c>
+      <c r="E7" t="s">
+        <v>3032</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H7">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8" t="s">
+        <v>3013</v>
+      </c>
+      <c r="D8" t="s">
+        <v>3023</v>
+      </c>
+      <c r="E8" t="s">
+        <v>3033</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H8">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>3014</v>
+      </c>
+      <c r="D9" t="s">
+        <v>3024</v>
+      </c>
+      <c r="E9" t="s">
+        <v>3034</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H9">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>1</v>
+      </c>
+      <c r="C10" t="s">
+        <v>3015</v>
+      </c>
+      <c r="D10" t="s">
+        <v>3025</v>
+      </c>
+      <c r="E10" t="s">
+        <v>3035</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H10">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>1</v>
+      </c>
+      <c r="C11" t="s">
+        <v>3016</v>
+      </c>
+      <c r="D11" t="s">
+        <v>3026</v>
+      </c>
+      <c r="E11" t="s">
+        <v>3036</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H11">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12">
+        <v>2</v>
+      </c>
+      <c r="C12" t="s">
+        <v>3007</v>
+      </c>
+      <c r="D12" t="s">
+        <v>3017</v>
+      </c>
+      <c r="E12" t="s">
+        <v>3027</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H12">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13">
+        <v>2</v>
+      </c>
+      <c r="C13" t="s">
+        <v>3008</v>
+      </c>
+      <c r="D13" t="s">
+        <v>3018</v>
+      </c>
+      <c r="E13" t="s">
+        <v>3028</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H13">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14">
+        <v>2</v>
+      </c>
+      <c r="C14" t="s">
+        <v>3009</v>
+      </c>
+      <c r="D14" t="s">
+        <v>3019</v>
+      </c>
+      <c r="E14" t="s">
+        <v>3029</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H14">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15">
+        <v>2</v>
+      </c>
+      <c r="C15" t="s">
+        <v>3010</v>
+      </c>
+      <c r="D15" t="s">
+        <v>3020</v>
+      </c>
+      <c r="E15" t="s">
+        <v>3030</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H15">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>3011</v>
+      </c>
+      <c r="D16" t="s">
+        <v>3021</v>
+      </c>
+      <c r="E16" t="s">
+        <v>3031</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H16">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17">
+        <v>2</v>
+      </c>
+      <c r="C17" t="s">
+        <v>3012</v>
+      </c>
+      <c r="D17" t="s">
+        <v>3022</v>
+      </c>
+      <c r="E17" t="s">
+        <v>3032</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H17">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>3013</v>
+      </c>
+      <c r="D18" t="s">
+        <v>3023</v>
+      </c>
+      <c r="E18" t="s">
+        <v>3033</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H18">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>3014</v>
+      </c>
+      <c r="D19" t="s">
+        <v>3024</v>
+      </c>
+      <c r="E19" t="s">
+        <v>3034</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H19">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20">
+        <v>2</v>
+      </c>
+      <c r="C20" t="s">
+        <v>3015</v>
+      </c>
+      <c r="D20" t="s">
+        <v>3025</v>
+      </c>
+      <c r="E20" t="s">
+        <v>3035</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H20">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>3016</v>
+      </c>
+      <c r="D21" t="s">
+        <v>3026</v>
+      </c>
+      <c r="E21" t="s">
+        <v>3036</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H21">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22">
+        <v>3</v>
+      </c>
+      <c r="C22" t="s">
+        <v>3007</v>
+      </c>
+      <c r="D22" t="s">
+        <v>3017</v>
+      </c>
+      <c r="E22" t="s">
+        <v>3027</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H22">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23">
+        <v>3</v>
+      </c>
+      <c r="C23" t="s">
+        <v>3008</v>
+      </c>
+      <c r="D23" t="s">
+        <v>3018</v>
+      </c>
+      <c r="E23" t="s">
+        <v>3028</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H23">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24">
+        <v>3</v>
+      </c>
+      <c r="C24" t="s">
+        <v>3009</v>
+      </c>
+      <c r="D24" t="s">
+        <v>3019</v>
+      </c>
+      <c r="E24" t="s">
+        <v>3029</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H24">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25">
+        <v>3</v>
+      </c>
+      <c r="C25" t="s">
+        <v>3010</v>
+      </c>
+      <c r="D25" t="s">
+        <v>3020</v>
+      </c>
+      <c r="E25" t="s">
+        <v>3030</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26">
+        <v>3</v>
+      </c>
+      <c r="C26" t="s">
+        <v>3011</v>
+      </c>
+      <c r="D26" t="s">
+        <v>3021</v>
+      </c>
+      <c r="E26" t="s">
+        <v>3031</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H26">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27">
+        <v>3</v>
+      </c>
+      <c r="C27" t="s">
+        <v>3012</v>
+      </c>
+      <c r="D27" t="s">
+        <v>3022</v>
+      </c>
+      <c r="E27" t="s">
+        <v>3032</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H27">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28">
+        <v>3</v>
+      </c>
+      <c r="C28" t="s">
+        <v>3013</v>
+      </c>
+      <c r="D28" t="s">
+        <v>3023</v>
+      </c>
+      <c r="E28" t="s">
+        <v>3033</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H28">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29">
+        <v>3</v>
+      </c>
+      <c r="C29" t="s">
+        <v>3014</v>
+      </c>
+      <c r="D29" t="s">
+        <v>3024</v>
+      </c>
+      <c r="E29" t="s">
+        <v>3034</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H29">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30">
+        <v>3</v>
+      </c>
+      <c r="C30" t="s">
+        <v>3015</v>
+      </c>
+      <c r="D30" t="s">
+        <v>3025</v>
+      </c>
+      <c r="E30" t="s">
+        <v>3035</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H30">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31">
+        <v>3</v>
+      </c>
+      <c r="C31" t="s">
+        <v>3016</v>
+      </c>
+      <c r="D31" t="s">
+        <v>3026</v>
+      </c>
+      <c r="E31" t="s">
+        <v>3036</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H31">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32">
+        <v>4</v>
+      </c>
+      <c r="C32" t="s">
+        <v>3007</v>
+      </c>
+      <c r="D32" t="s">
+        <v>3017</v>
+      </c>
+      <c r="E32" t="s">
+        <v>3027</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H32">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33">
+        <v>4</v>
+      </c>
+      <c r="C33" t="s">
+        <v>3008</v>
+      </c>
+      <c r="D33" t="s">
+        <v>3018</v>
+      </c>
+      <c r="E33" t="s">
+        <v>3028</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H33">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34">
+        <v>4</v>
+      </c>
+      <c r="C34" t="s">
+        <v>3009</v>
+      </c>
+      <c r="D34" t="s">
+        <v>3019</v>
+      </c>
+      <c r="E34" t="s">
+        <v>3029</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H34">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35">
+        <v>4</v>
+      </c>
+      <c r="C35" t="s">
+        <v>3010</v>
+      </c>
+      <c r="D35" t="s">
+        <v>3020</v>
+      </c>
+      <c r="E35" t="s">
+        <v>3030</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G35" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H35">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36">
+        <v>4</v>
+      </c>
+      <c r="C36" t="s">
+        <v>3011</v>
+      </c>
+      <c r="D36" t="s">
+        <v>3021</v>
+      </c>
+      <c r="E36" t="s">
+        <v>3031</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H36">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37">
+        <v>4</v>
+      </c>
+      <c r="C37" t="s">
+        <v>3012</v>
+      </c>
+      <c r="D37" t="s">
+        <v>3022</v>
+      </c>
+      <c r="E37" t="s">
+        <v>3032</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H37">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38">
+        <v>4</v>
+      </c>
+      <c r="C38" t="s">
+        <v>3013</v>
+      </c>
+      <c r="D38" t="s">
+        <v>3023</v>
+      </c>
+      <c r="E38" t="s">
+        <v>3033</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H38">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>38</v>
+      </c>
+      <c r="B39">
+        <v>4</v>
+      </c>
+      <c r="C39" t="s">
+        <v>3014</v>
+      </c>
+      <c r="D39" t="s">
+        <v>3024</v>
+      </c>
+      <c r="E39" t="s">
+        <v>3034</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H39">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>39</v>
+      </c>
+      <c r="B40">
+        <v>4</v>
+      </c>
+      <c r="C40" t="s">
+        <v>3015</v>
+      </c>
+      <c r="D40" t="s">
+        <v>3025</v>
+      </c>
+      <c r="E40" t="s">
+        <v>3035</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H40">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41">
+        <v>4</v>
+      </c>
+      <c r="C41" t="s">
+        <v>3016</v>
+      </c>
+      <c r="D41" t="s">
+        <v>3026</v>
+      </c>
+      <c r="E41" t="s">
+        <v>3036</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H41">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A42">
+        <v>41</v>
+      </c>
+      <c r="B42">
+        <v>5</v>
+      </c>
+      <c r="C42" t="s">
+        <v>3007</v>
+      </c>
+      <c r="D42" t="s">
+        <v>3017</v>
+      </c>
+      <c r="E42" t="s">
+        <v>3027</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H42">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A43">
+        <v>42</v>
+      </c>
+      <c r="B43">
+        <v>5</v>
+      </c>
+      <c r="C43" t="s">
+        <v>3008</v>
+      </c>
+      <c r="D43" t="s">
+        <v>3018</v>
+      </c>
+      <c r="E43" t="s">
+        <v>3028</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G43" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H43">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A44">
+        <v>43</v>
+      </c>
+      <c r="B44">
+        <v>5</v>
+      </c>
+      <c r="C44" t="s">
+        <v>3009</v>
+      </c>
+      <c r="D44" t="s">
+        <v>3019</v>
+      </c>
+      <c r="E44" t="s">
+        <v>3029</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G44" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H44">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <v>44</v>
+      </c>
+      <c r="B45">
+        <v>5</v>
+      </c>
+      <c r="C45" t="s">
+        <v>3010</v>
+      </c>
+      <c r="D45" t="s">
+        <v>3020</v>
+      </c>
+      <c r="E45" t="s">
+        <v>3030</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G45" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H45">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A46">
+        <v>45</v>
+      </c>
+      <c r="B46">
+        <v>5</v>
+      </c>
+      <c r="C46" t="s">
+        <v>3011</v>
+      </c>
+      <c r="D46" t="s">
+        <v>3021</v>
+      </c>
+      <c r="E46" t="s">
+        <v>3031</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G46" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H46">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A47">
+        <v>46</v>
+      </c>
+      <c r="B47">
+        <v>5</v>
+      </c>
+      <c r="C47" t="s">
+        <v>3012</v>
+      </c>
+      <c r="D47" t="s">
+        <v>3022</v>
+      </c>
+      <c r="E47" t="s">
+        <v>3032</v>
+      </c>
+      <c r="F47" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G47" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H47">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A48">
+        <v>47</v>
+      </c>
+      <c r="B48">
+        <v>5</v>
+      </c>
+      <c r="C48" t="s">
+        <v>3013</v>
+      </c>
+      <c r="D48" t="s">
+        <v>3023</v>
+      </c>
+      <c r="E48" t="s">
+        <v>3033</v>
+      </c>
+      <c r="F48" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G48" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H48">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A49">
+        <v>48</v>
+      </c>
+      <c r="B49">
+        <v>5</v>
+      </c>
+      <c r="C49" t="s">
+        <v>3014</v>
+      </c>
+      <c r="D49" t="s">
+        <v>3024</v>
+      </c>
+      <c r="E49" t="s">
+        <v>3034</v>
+      </c>
+      <c r="F49" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G49" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H49">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A50">
+        <v>49</v>
+      </c>
+      <c r="B50">
+        <v>5</v>
+      </c>
+      <c r="C50" t="s">
+        <v>3015</v>
+      </c>
+      <c r="D50" t="s">
+        <v>3025</v>
+      </c>
+      <c r="E50" t="s">
+        <v>3035</v>
+      </c>
+      <c r="F50" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G50" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H50">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A51">
+        <v>50</v>
+      </c>
+      <c r="B51">
+        <v>5</v>
+      </c>
+      <c r="C51" t="s">
+        <v>3016</v>
+      </c>
+      <c r="D51" t="s">
+        <v>3026</v>
+      </c>
+      <c r="E51" t="s">
+        <v>3036</v>
+      </c>
+      <c r="F51" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G51" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H51">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A52">
+        <v>51</v>
+      </c>
+      <c r="B52">
+        <v>6</v>
+      </c>
+      <c r="C52" t="s">
+        <v>3007</v>
+      </c>
+      <c r="D52" t="s">
+        <v>3017</v>
+      </c>
+      <c r="E52" t="s">
+        <v>3027</v>
+      </c>
+      <c r="F52" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G52" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H52">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A53">
+        <v>52</v>
+      </c>
+      <c r="B53">
+        <v>6</v>
+      </c>
+      <c r="C53" t="s">
+        <v>3008</v>
+      </c>
+      <c r="D53" t="s">
+        <v>3018</v>
+      </c>
+      <c r="E53" t="s">
+        <v>3028</v>
+      </c>
+      <c r="F53" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G53" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H53">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A54">
+        <v>53</v>
+      </c>
+      <c r="B54">
+        <v>6</v>
+      </c>
+      <c r="C54" t="s">
+        <v>3009</v>
+      </c>
+      <c r="D54" t="s">
+        <v>3019</v>
+      </c>
+      <c r="E54" t="s">
+        <v>3029</v>
+      </c>
+      <c r="F54" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G54" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H54">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A55">
+        <v>54</v>
+      </c>
+      <c r="B55">
+        <v>6</v>
+      </c>
+      <c r="C55" t="s">
+        <v>3010</v>
+      </c>
+      <c r="D55" t="s">
+        <v>3020</v>
+      </c>
+      <c r="E55" t="s">
+        <v>3030</v>
+      </c>
+      <c r="F55" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G55" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H55">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A56">
+        <v>55</v>
+      </c>
+      <c r="B56">
+        <v>6</v>
+      </c>
+      <c r="C56" t="s">
+        <v>3011</v>
+      </c>
+      <c r="D56" t="s">
+        <v>3021</v>
+      </c>
+      <c r="E56" t="s">
+        <v>3031</v>
+      </c>
+      <c r="F56" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G56" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H56">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A57">
+        <v>56</v>
+      </c>
+      <c r="B57">
+        <v>6</v>
+      </c>
+      <c r="C57" t="s">
+        <v>3012</v>
+      </c>
+      <c r="D57" t="s">
+        <v>3022</v>
+      </c>
+      <c r="E57" t="s">
+        <v>3032</v>
+      </c>
+      <c r="F57" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G57" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H57">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A58">
+        <v>57</v>
+      </c>
+      <c r="B58">
+        <v>6</v>
+      </c>
+      <c r="C58" t="s">
+        <v>3013</v>
+      </c>
+      <c r="D58" t="s">
+        <v>3023</v>
+      </c>
+      <c r="E58" t="s">
+        <v>3033</v>
+      </c>
+      <c r="F58" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G58" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H58">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A59">
+        <v>58</v>
+      </c>
+      <c r="B59">
+        <v>6</v>
+      </c>
+      <c r="C59" t="s">
+        <v>3014</v>
+      </c>
+      <c r="D59" t="s">
+        <v>3024</v>
+      </c>
+      <c r="E59" t="s">
+        <v>3034</v>
+      </c>
+      <c r="F59" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G59" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H59">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A60">
+        <v>59</v>
+      </c>
+      <c r="B60">
+        <v>6</v>
+      </c>
+      <c r="C60" t="s">
+        <v>3015</v>
+      </c>
+      <c r="D60" t="s">
+        <v>3025</v>
+      </c>
+      <c r="E60" t="s">
+        <v>3035</v>
+      </c>
+      <c r="F60" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G60" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H60">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A61">
+        <v>60</v>
+      </c>
+      <c r="B61">
+        <v>6</v>
+      </c>
+      <c r="C61" t="s">
+        <v>3016</v>
+      </c>
+      <c r="D61" t="s">
+        <v>3026</v>
+      </c>
+      <c r="E61" t="s">
+        <v>3036</v>
+      </c>
+      <c r="F61" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G61" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H61">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A62">
+        <v>61</v>
+      </c>
+      <c r="B62">
+        <v>7</v>
+      </c>
+      <c r="C62" t="s">
+        <v>3007</v>
+      </c>
+      <c r="D62" t="s">
+        <v>3017</v>
+      </c>
+      <c r="E62" t="s">
+        <v>3027</v>
+      </c>
+      <c r="F62" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G62" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H62">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A63">
+        <v>62</v>
+      </c>
+      <c r="B63">
+        <v>7</v>
+      </c>
+      <c r="C63" t="s">
+        <v>3008</v>
+      </c>
+      <c r="D63" t="s">
+        <v>3018</v>
+      </c>
+      <c r="E63" t="s">
+        <v>3028</v>
+      </c>
+      <c r="F63" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G63" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H63">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A64">
+        <v>63</v>
+      </c>
+      <c r="B64">
+        <v>7</v>
+      </c>
+      <c r="C64" t="s">
+        <v>3009</v>
+      </c>
+      <c r="D64" t="s">
+        <v>3019</v>
+      </c>
+      <c r="E64" t="s">
+        <v>3029</v>
+      </c>
+      <c r="F64" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G64" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H64">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A65">
+        <v>64</v>
+      </c>
+      <c r="B65">
+        <v>7</v>
+      </c>
+      <c r="C65" t="s">
+        <v>3010</v>
+      </c>
+      <c r="D65" t="s">
+        <v>3020</v>
+      </c>
+      <c r="E65" t="s">
+        <v>3030</v>
+      </c>
+      <c r="F65" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G65" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H65">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A66">
+        <v>65</v>
+      </c>
+      <c r="B66">
+        <v>7</v>
+      </c>
+      <c r="C66" t="s">
+        <v>3011</v>
+      </c>
+      <c r="D66" t="s">
+        <v>3021</v>
+      </c>
+      <c r="E66" t="s">
+        <v>3031</v>
+      </c>
+      <c r="F66" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G66" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H66">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A67">
+        <v>66</v>
+      </c>
+      <c r="B67">
+        <v>7</v>
+      </c>
+      <c r="C67" t="s">
+        <v>3012</v>
+      </c>
+      <c r="D67" t="s">
+        <v>3022</v>
+      </c>
+      <c r="E67" t="s">
+        <v>3032</v>
+      </c>
+      <c r="F67" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G67" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H67">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A68">
+        <v>67</v>
+      </c>
+      <c r="B68">
+        <v>7</v>
+      </c>
+      <c r="C68" t="s">
+        <v>3013</v>
+      </c>
+      <c r="D68" t="s">
+        <v>3023</v>
+      </c>
+      <c r="E68" t="s">
+        <v>3033</v>
+      </c>
+      <c r="F68" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G68" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H68">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A69">
+        <v>68</v>
+      </c>
+      <c r="B69">
+        <v>7</v>
+      </c>
+      <c r="C69" t="s">
+        <v>3014</v>
+      </c>
+      <c r="D69" t="s">
+        <v>3024</v>
+      </c>
+      <c r="E69" t="s">
+        <v>3034</v>
+      </c>
+      <c r="F69" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G69" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H69">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A70">
+        <v>69</v>
+      </c>
+      <c r="B70">
+        <v>7</v>
+      </c>
+      <c r="C70" t="s">
+        <v>3015</v>
+      </c>
+      <c r="D70" t="s">
+        <v>3025</v>
+      </c>
+      <c r="E70" t="s">
+        <v>3035</v>
+      </c>
+      <c r="F70" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G70" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H70">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A71">
+        <v>70</v>
+      </c>
+      <c r="B71">
+        <v>7</v>
+      </c>
+      <c r="C71" t="s">
+        <v>3016</v>
+      </c>
+      <c r="D71" t="s">
+        <v>3026</v>
+      </c>
+      <c r="E71" t="s">
+        <v>3036</v>
+      </c>
+      <c r="F71" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G71" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H71">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A72">
+        <v>71</v>
+      </c>
+      <c r="B72">
+        <v>8</v>
+      </c>
+      <c r="C72" t="s">
+        <v>3007</v>
+      </c>
+      <c r="D72" t="s">
+        <v>3017</v>
+      </c>
+      <c r="E72" t="s">
+        <v>3027</v>
+      </c>
+      <c r="F72" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G72" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H72">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A73">
+        <v>72</v>
+      </c>
+      <c r="B73">
+        <v>8</v>
+      </c>
+      <c r="C73" t="s">
+        <v>3008</v>
+      </c>
+      <c r="D73" t="s">
+        <v>3018</v>
+      </c>
+      <c r="E73" t="s">
+        <v>3028</v>
+      </c>
+      <c r="F73" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G73" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H73">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A74">
+        <v>73</v>
+      </c>
+      <c r="B74">
+        <v>8</v>
+      </c>
+      <c r="C74" t="s">
+        <v>3009</v>
+      </c>
+      <c r="D74" t="s">
+        <v>3019</v>
+      </c>
+      <c r="E74" t="s">
+        <v>3029</v>
+      </c>
+      <c r="F74" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G74" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H74">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A75">
+        <v>74</v>
+      </c>
+      <c r="B75">
+        <v>8</v>
+      </c>
+      <c r="C75" t="s">
+        <v>3010</v>
+      </c>
+      <c r="D75" t="s">
+        <v>3020</v>
+      </c>
+      <c r="E75" t="s">
+        <v>3030</v>
+      </c>
+      <c r="F75" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G75" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H75">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A76">
+        <v>75</v>
+      </c>
+      <c r="B76">
+        <v>8</v>
+      </c>
+      <c r="C76" t="s">
+        <v>3011</v>
+      </c>
+      <c r="D76" t="s">
+        <v>3021</v>
+      </c>
+      <c r="E76" t="s">
+        <v>3031</v>
+      </c>
+      <c r="F76" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G76" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H76">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A77">
+        <v>76</v>
+      </c>
+      <c r="B77">
+        <v>8</v>
+      </c>
+      <c r="C77" t="s">
+        <v>3012</v>
+      </c>
+      <c r="D77" t="s">
+        <v>3022</v>
+      </c>
+      <c r="E77" t="s">
+        <v>3032</v>
+      </c>
+      <c r="F77" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G77" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H77">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A78">
+        <v>77</v>
+      </c>
+      <c r="B78">
+        <v>8</v>
+      </c>
+      <c r="C78" t="s">
+        <v>3013</v>
+      </c>
+      <c r="D78" t="s">
+        <v>3023</v>
+      </c>
+      <c r="E78" t="s">
+        <v>3033</v>
+      </c>
+      <c r="F78" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G78" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H78">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A79">
+        <v>78</v>
+      </c>
+      <c r="B79">
+        <v>8</v>
+      </c>
+      <c r="C79" t="s">
+        <v>3014</v>
+      </c>
+      <c r="D79" t="s">
+        <v>3024</v>
+      </c>
+      <c r="E79" t="s">
+        <v>3034</v>
+      </c>
+      <c r="F79" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G79" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H79">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A80">
+        <v>79</v>
+      </c>
+      <c r="B80">
+        <v>8</v>
+      </c>
+      <c r="C80" t="s">
+        <v>3015</v>
+      </c>
+      <c r="D80" t="s">
+        <v>3025</v>
+      </c>
+      <c r="E80" t="s">
+        <v>3035</v>
+      </c>
+      <c r="F80" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G80" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H80">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A81">
+        <v>80</v>
+      </c>
+      <c r="B81">
+        <v>8</v>
+      </c>
+      <c r="C81" t="s">
+        <v>3016</v>
+      </c>
+      <c r="D81" t="s">
+        <v>3026</v>
+      </c>
+      <c r="E81" t="s">
+        <v>3036</v>
+      </c>
+      <c r="F81" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G81" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H81">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A82">
+        <v>81</v>
+      </c>
+      <c r="B82">
+        <v>9</v>
+      </c>
+      <c r="C82" t="s">
+        <v>3007</v>
+      </c>
+      <c r="D82" t="s">
+        <v>3017</v>
+      </c>
+      <c r="E82" t="s">
+        <v>3027</v>
+      </c>
+      <c r="F82" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G82" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H82">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A83">
+        <v>82</v>
+      </c>
+      <c r="B83">
+        <v>9</v>
+      </c>
+      <c r="C83" t="s">
+        <v>3008</v>
+      </c>
+      <c r="D83" t="s">
+        <v>3018</v>
+      </c>
+      <c r="E83" t="s">
+        <v>3028</v>
+      </c>
+      <c r="F83" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G83" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H83">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A84">
+        <v>83</v>
+      </c>
+      <c r="B84">
+        <v>9</v>
+      </c>
+      <c r="C84" t="s">
+        <v>3009</v>
+      </c>
+      <c r="D84" t="s">
+        <v>3019</v>
+      </c>
+      <c r="E84" t="s">
+        <v>3029</v>
+      </c>
+      <c r="F84" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G84" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H84">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A85">
+        <v>84</v>
+      </c>
+      <c r="B85">
+        <v>9</v>
+      </c>
+      <c r="C85" t="s">
+        <v>3010</v>
+      </c>
+      <c r="D85" t="s">
+        <v>3020</v>
+      </c>
+      <c r="E85" t="s">
+        <v>3030</v>
+      </c>
+      <c r="F85" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G85" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H85">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A86">
+        <v>85</v>
+      </c>
+      <c r="B86">
+        <v>9</v>
+      </c>
+      <c r="C86" t="s">
+        <v>3011</v>
+      </c>
+      <c r="D86" t="s">
+        <v>3021</v>
+      </c>
+      <c r="E86" t="s">
+        <v>3031</v>
+      </c>
+      <c r="F86" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G86" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H86">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A87">
+        <v>86</v>
+      </c>
+      <c r="B87">
+        <v>9</v>
+      </c>
+      <c r="C87" t="s">
+        <v>3012</v>
+      </c>
+      <c r="D87" t="s">
+        <v>3022</v>
+      </c>
+      <c r="E87" t="s">
+        <v>3032</v>
+      </c>
+      <c r="F87" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G87" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H87">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A88">
+        <v>87</v>
+      </c>
+      <c r="B88">
+        <v>9</v>
+      </c>
+      <c r="C88" t="s">
+        <v>3013</v>
+      </c>
+      <c r="D88" t="s">
+        <v>3023</v>
+      </c>
+      <c r="E88" t="s">
+        <v>3033</v>
+      </c>
+      <c r="F88" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G88" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H88">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A89">
+        <v>88</v>
+      </c>
+      <c r="B89">
+        <v>9</v>
+      </c>
+      <c r="C89" t="s">
+        <v>3014</v>
+      </c>
+      <c r="D89" t="s">
+        <v>3024</v>
+      </c>
+      <c r="E89" t="s">
+        <v>3034</v>
+      </c>
+      <c r="F89" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G89" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H89">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A90">
+        <v>89</v>
+      </c>
+      <c r="B90">
+        <v>9</v>
+      </c>
+      <c r="C90" t="s">
+        <v>3015</v>
+      </c>
+      <c r="D90" t="s">
+        <v>3025</v>
+      </c>
+      <c r="E90" t="s">
+        <v>3035</v>
+      </c>
+      <c r="F90" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G90" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H90">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A91">
+        <v>90</v>
+      </c>
+      <c r="B91">
+        <v>9</v>
+      </c>
+      <c r="C91" t="s">
+        <v>3016</v>
+      </c>
+      <c r="D91" t="s">
+        <v>3026</v>
+      </c>
+      <c r="E91" t="s">
+        <v>3036</v>
+      </c>
+      <c r="F91" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G91" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H91">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A92">
+        <v>91</v>
+      </c>
+      <c r="B92">
+        <v>10</v>
+      </c>
+      <c r="C92" t="s">
+        <v>3007</v>
+      </c>
+      <c r="D92" t="s">
+        <v>3017</v>
+      </c>
+      <c r="E92" t="s">
+        <v>3027</v>
+      </c>
+      <c r="F92" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G92" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H92">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A93">
+        <v>92</v>
+      </c>
+      <c r="B93">
+        <v>10</v>
+      </c>
+      <c r="C93" t="s">
+        <v>3008</v>
+      </c>
+      <c r="D93" t="s">
+        <v>3018</v>
+      </c>
+      <c r="E93" t="s">
+        <v>3028</v>
+      </c>
+      <c r="F93" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G93" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H93">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A94">
+        <v>93</v>
+      </c>
+      <c r="B94">
+        <v>10</v>
+      </c>
+      <c r="C94" t="s">
+        <v>3009</v>
+      </c>
+      <c r="D94" t="s">
+        <v>3019</v>
+      </c>
+      <c r="E94" t="s">
+        <v>3029</v>
+      </c>
+      <c r="F94" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G94" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H94">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A95">
+        <v>94</v>
+      </c>
+      <c r="B95">
+        <v>10</v>
+      </c>
+      <c r="C95" t="s">
+        <v>3010</v>
+      </c>
+      <c r="D95" t="s">
+        <v>3020</v>
+      </c>
+      <c r="E95" t="s">
+        <v>3030</v>
+      </c>
+      <c r="F95" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G95" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H95">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A96">
+        <v>95</v>
+      </c>
+      <c r="B96">
+        <v>10</v>
+      </c>
+      <c r="C96" t="s">
+        <v>3011</v>
+      </c>
+      <c r="D96" t="s">
+        <v>3021</v>
+      </c>
+      <c r="E96" t="s">
+        <v>3031</v>
+      </c>
+      <c r="F96" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G96" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H96">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A97">
+        <v>96</v>
+      </c>
+      <c r="B97">
+        <v>10</v>
+      </c>
+      <c r="C97" t="s">
+        <v>3012</v>
+      </c>
+      <c r="D97" t="s">
+        <v>3022</v>
+      </c>
+      <c r="E97" t="s">
+        <v>3032</v>
+      </c>
+      <c r="F97" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G97" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H97">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A98">
+        <v>97</v>
+      </c>
+      <c r="B98">
+        <v>10</v>
+      </c>
+      <c r="C98" t="s">
+        <v>3013</v>
+      </c>
+      <c r="D98" t="s">
+        <v>3023</v>
+      </c>
+      <c r="E98" t="s">
+        <v>3033</v>
+      </c>
+      <c r="F98" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G98" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H98">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A99">
+        <v>98</v>
+      </c>
+      <c r="B99">
+        <v>10</v>
+      </c>
+      <c r="C99" t="s">
+        <v>3014</v>
+      </c>
+      <c r="D99" t="s">
+        <v>3024</v>
+      </c>
+      <c r="E99" t="s">
+        <v>3034</v>
+      </c>
+      <c r="F99" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G99" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H99">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="100" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A100">
+        <v>99</v>
+      </c>
+      <c r="B100">
+        <v>10</v>
+      </c>
+      <c r="C100" t="s">
+        <v>3015</v>
+      </c>
+      <c r="D100" t="s">
+        <v>3025</v>
+      </c>
+      <c r="E100" t="s">
+        <v>3035</v>
+      </c>
+      <c r="F100" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G100" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H100">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="101" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A101">
+        <v>100</v>
+      </c>
+      <c r="B101">
+        <v>10</v>
+      </c>
+      <c r="C101" t="s">
+        <v>3016</v>
+      </c>
+      <c r="D101" t="s">
+        <v>3026</v>
+      </c>
+      <c r="E101" t="s">
+        <v>3036</v>
+      </c>
+      <c r="F101" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G101" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H101">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="102" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A102">
+        <v>101</v>
+      </c>
+      <c r="B102">
+        <v>11</v>
+      </c>
+      <c r="C102" t="s">
+        <v>3007</v>
+      </c>
+      <c r="D102" t="s">
+        <v>3017</v>
+      </c>
+      <c r="E102" t="s">
+        <v>3027</v>
+      </c>
+      <c r="F102" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G102" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H102">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="103" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A103">
+        <v>102</v>
+      </c>
+      <c r="B103">
+        <v>11</v>
+      </c>
+      <c r="C103" t="s">
+        <v>3008</v>
+      </c>
+      <c r="D103" t="s">
+        <v>3018</v>
+      </c>
+      <c r="E103" t="s">
+        <v>3028</v>
+      </c>
+      <c r="F103" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G103" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H103">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="104" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A104">
+        <v>103</v>
+      </c>
+      <c r="B104">
+        <v>11</v>
+      </c>
+      <c r="C104" t="s">
+        <v>3009</v>
+      </c>
+      <c r="D104" t="s">
+        <v>3019</v>
+      </c>
+      <c r="E104" t="s">
+        <v>3029</v>
+      </c>
+      <c r="F104" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G104" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H104">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="105" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A105">
+        <v>104</v>
+      </c>
+      <c r="B105">
+        <v>11</v>
+      </c>
+      <c r="C105" t="s">
+        <v>3010</v>
+      </c>
+      <c r="D105" t="s">
+        <v>3020</v>
+      </c>
+      <c r="E105" t="s">
+        <v>3030</v>
+      </c>
+      <c r="F105" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G105" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H105">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="106" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A106">
+        <v>105</v>
+      </c>
+      <c r="B106">
+        <v>11</v>
+      </c>
+      <c r="C106" t="s">
+        <v>3011</v>
+      </c>
+      <c r="D106" t="s">
+        <v>3021</v>
+      </c>
+      <c r="E106" t="s">
+        <v>3031</v>
+      </c>
+      <c r="F106" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G106" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H106">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="107" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A107">
+        <v>106</v>
+      </c>
+      <c r="B107">
+        <v>11</v>
+      </c>
+      <c r="C107" t="s">
+        <v>3012</v>
+      </c>
+      <c r="D107" t="s">
+        <v>3022</v>
+      </c>
+      <c r="E107" t="s">
+        <v>3032</v>
+      </c>
+      <c r="F107" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G107" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H107">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="108" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A108">
+        <v>107</v>
+      </c>
+      <c r="B108">
+        <v>11</v>
+      </c>
+      <c r="C108" t="s">
+        <v>3013</v>
+      </c>
+      <c r="D108" t="s">
+        <v>3023</v>
+      </c>
+      <c r="E108" t="s">
+        <v>3033</v>
+      </c>
+      <c r="F108" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G108" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H108">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="109" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A109">
+        <v>108</v>
+      </c>
+      <c r="B109">
+        <v>11</v>
+      </c>
+      <c r="C109" t="s">
+        <v>3014</v>
+      </c>
+      <c r="D109" t="s">
+        <v>3024</v>
+      </c>
+      <c r="E109" t="s">
+        <v>3034</v>
+      </c>
+      <c r="F109" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G109" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H109">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="110" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A110">
+        <v>109</v>
+      </c>
+      <c r="B110">
+        <v>11</v>
+      </c>
+      <c r="C110" t="s">
+        <v>3015</v>
+      </c>
+      <c r="D110" t="s">
+        <v>3025</v>
+      </c>
+      <c r="E110" t="s">
+        <v>3035</v>
+      </c>
+      <c r="F110" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G110" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H110">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="111" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A111">
+        <v>110</v>
+      </c>
+      <c r="B111">
+        <v>11</v>
+      </c>
+      <c r="C111" t="s">
+        <v>3016</v>
+      </c>
+      <c r="D111" t="s">
+        <v>3026</v>
+      </c>
+      <c r="E111" t="s">
+        <v>3036</v>
+      </c>
+      <c r="F111" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G111" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H111">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="112" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A112">
+        <v>111</v>
+      </c>
+      <c r="B112">
+        <v>12</v>
+      </c>
+      <c r="C112" t="s">
+        <v>3007</v>
+      </c>
+      <c r="D112" t="s">
+        <v>3017</v>
+      </c>
+      <c r="E112" t="s">
+        <v>3027</v>
+      </c>
+      <c r="F112" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G112" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H112">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="113" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A113">
+        <v>112</v>
+      </c>
+      <c r="B113">
+        <v>12</v>
+      </c>
+      <c r="C113" t="s">
+        <v>3008</v>
+      </c>
+      <c r="D113" t="s">
+        <v>3018</v>
+      </c>
+      <c r="E113" t="s">
+        <v>3028</v>
+      </c>
+      <c r="F113" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G113" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H113">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="114" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A114">
+        <v>113</v>
+      </c>
+      <c r="B114">
+        <v>12</v>
+      </c>
+      <c r="C114" t="s">
+        <v>3009</v>
+      </c>
+      <c r="D114" t="s">
+        <v>3019</v>
+      </c>
+      <c r="E114" t="s">
+        <v>3029</v>
+      </c>
+      <c r="F114" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G114" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H114">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="115" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A115">
+        <v>114</v>
+      </c>
+      <c r="B115">
+        <v>12</v>
+      </c>
+      <c r="C115" t="s">
+        <v>3010</v>
+      </c>
+      <c r="D115" t="s">
+        <v>3020</v>
+      </c>
+      <c r="E115" t="s">
+        <v>3030</v>
+      </c>
+      <c r="F115" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G115" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H115">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="116" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A116">
+        <v>115</v>
+      </c>
+      <c r="B116">
+        <v>12</v>
+      </c>
+      <c r="C116" t="s">
+        <v>3011</v>
+      </c>
+      <c r="D116" t="s">
+        <v>3021</v>
+      </c>
+      <c r="E116" t="s">
+        <v>3031</v>
+      </c>
+      <c r="F116" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G116" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H116">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="117" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A117">
+        <v>116</v>
+      </c>
+      <c r="B117">
+        <v>12</v>
+      </c>
+      <c r="C117" t="s">
+        <v>3012</v>
+      </c>
+      <c r="D117" t="s">
+        <v>3022</v>
+      </c>
+      <c r="E117" t="s">
+        <v>3032</v>
+      </c>
+      <c r="F117" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G117" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H117">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="118" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A118">
+        <v>117</v>
+      </c>
+      <c r="B118">
+        <v>12</v>
+      </c>
+      <c r="C118" t="s">
+        <v>3013</v>
+      </c>
+      <c r="D118" t="s">
+        <v>3023</v>
+      </c>
+      <c r="E118" t="s">
+        <v>3033</v>
+      </c>
+      <c r="F118" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G118" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H118">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="119" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A119">
+        <v>118</v>
+      </c>
+      <c r="B119">
+        <v>12</v>
+      </c>
+      <c r="C119" t="s">
+        <v>3014</v>
+      </c>
+      <c r="D119" t="s">
+        <v>3024</v>
+      </c>
+      <c r="E119" t="s">
+        <v>3034</v>
+      </c>
+      <c r="F119" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G119" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H119">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="120" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A120">
+        <v>119</v>
+      </c>
+      <c r="B120">
+        <v>12</v>
+      </c>
+      <c r="C120" t="s">
+        <v>3015</v>
+      </c>
+      <c r="D120" t="s">
+        <v>3025</v>
+      </c>
+      <c r="E120" t="s">
+        <v>3035</v>
+      </c>
+      <c r="F120" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G120" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H120">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="121" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A121">
+        <v>120</v>
+      </c>
+      <c r="B121">
+        <v>12</v>
+      </c>
+      <c r="C121" t="s">
+        <v>3016</v>
+      </c>
+      <c r="D121" t="s">
+        <v>3026</v>
+      </c>
+      <c r="E121" t="s">
+        <v>3036</v>
+      </c>
+      <c r="F121" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G121" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H121">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="122" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A122">
+        <v>121</v>
+      </c>
+      <c r="B122">
+        <v>13</v>
+      </c>
+      <c r="C122" t="s">
+        <v>3007</v>
+      </c>
+      <c r="D122" t="s">
+        <v>3017</v>
+      </c>
+      <c r="E122" t="s">
+        <v>3027</v>
+      </c>
+      <c r="F122" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G122" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H122">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="123" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A123">
+        <v>122</v>
+      </c>
+      <c r="B123">
+        <v>13</v>
+      </c>
+      <c r="C123" t="s">
+        <v>3008</v>
+      </c>
+      <c r="D123" t="s">
+        <v>3018</v>
+      </c>
+      <c r="E123" t="s">
+        <v>3028</v>
+      </c>
+      <c r="F123" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G123" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H123">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="124" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A124">
+        <v>123</v>
+      </c>
+      <c r="B124">
+        <v>13</v>
+      </c>
+      <c r="C124" t="s">
+        <v>3009</v>
+      </c>
+      <c r="D124" t="s">
+        <v>3019</v>
+      </c>
+      <c r="E124" t="s">
+        <v>3029</v>
+      </c>
+      <c r="F124" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G124" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H124">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="125" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A125">
+        <v>124</v>
+      </c>
+      <c r="B125">
+        <v>13</v>
+      </c>
+      <c r="C125" t="s">
+        <v>3010</v>
+      </c>
+      <c r="D125" t="s">
+        <v>3020</v>
+      </c>
+      <c r="E125" t="s">
+        <v>3030</v>
+      </c>
+      <c r="F125" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G125" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H125">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="126" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A126">
+        <v>125</v>
+      </c>
+      <c r="B126">
+        <v>13</v>
+      </c>
+      <c r="C126" t="s">
+        <v>3011</v>
+      </c>
+      <c r="D126" t="s">
+        <v>3021</v>
+      </c>
+      <c r="E126" t="s">
+        <v>3031</v>
+      </c>
+      <c r="F126" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G126" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H126">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="127" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A127">
+        <v>126</v>
+      </c>
+      <c r="B127">
+        <v>13</v>
+      </c>
+      <c r="C127" t="s">
+        <v>3012</v>
+      </c>
+      <c r="D127" t="s">
+        <v>3022</v>
+      </c>
+      <c r="E127" t="s">
+        <v>3032</v>
+      </c>
+      <c r="F127" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G127" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H127">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="128" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A128">
+        <v>127</v>
+      </c>
+      <c r="B128">
+        <v>13</v>
+      </c>
+      <c r="C128" t="s">
+        <v>3013</v>
+      </c>
+      <c r="D128" t="s">
+        <v>3023</v>
+      </c>
+      <c r="E128" t="s">
+        <v>3033</v>
+      </c>
+      <c r="F128" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G128" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H128">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="129" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A129">
+        <v>128</v>
+      </c>
+      <c r="B129">
+        <v>13</v>
+      </c>
+      <c r="C129" t="s">
+        <v>3014</v>
+      </c>
+      <c r="D129" t="s">
+        <v>3024</v>
+      </c>
+      <c r="E129" t="s">
+        <v>3034</v>
+      </c>
+      <c r="F129" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G129" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H129">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="130" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A130">
+        <v>129</v>
+      </c>
+      <c r="B130">
+        <v>13</v>
+      </c>
+      <c r="C130" t="s">
+        <v>3015</v>
+      </c>
+      <c r="D130" t="s">
+        <v>3025</v>
+      </c>
+      <c r="E130" t="s">
+        <v>3035</v>
+      </c>
+      <c r="F130" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G130" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H130">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="131" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A131">
+        <v>130</v>
+      </c>
+      <c r="B131">
+        <v>13</v>
+      </c>
+      <c r="C131" t="s">
+        <v>3016</v>
+      </c>
+      <c r="D131" t="s">
+        <v>3026</v>
+      </c>
+      <c r="E131" t="s">
+        <v>3036</v>
+      </c>
+      <c r="F131" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G131" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H131">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="132" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A132">
+        <v>131</v>
+      </c>
+      <c r="B132">
+        <v>14</v>
+      </c>
+      <c r="C132" t="s">
+        <v>3007</v>
+      </c>
+      <c r="D132" t="s">
+        <v>3017</v>
+      </c>
+      <c r="E132" t="s">
+        <v>3027</v>
+      </c>
+      <c r="F132" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G132" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H132">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="133" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A133">
+        <v>132</v>
+      </c>
+      <c r="B133">
+        <v>14</v>
+      </c>
+      <c r="C133" t="s">
+        <v>3008</v>
+      </c>
+      <c r="D133" t="s">
+        <v>3018</v>
+      </c>
+      <c r="E133" t="s">
+        <v>3028</v>
+      </c>
+      <c r="F133" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G133" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H133">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="134" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A134">
+        <v>133</v>
+      </c>
+      <c r="B134">
+        <v>14</v>
+      </c>
+      <c r="C134" t="s">
+        <v>3009</v>
+      </c>
+      <c r="D134" t="s">
+        <v>3019</v>
+      </c>
+      <c r="E134" t="s">
+        <v>3029</v>
+      </c>
+      <c r="F134" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G134" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H134">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="135" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A135">
+        <v>134</v>
+      </c>
+      <c r="B135">
+        <v>14</v>
+      </c>
+      <c r="C135" t="s">
+        <v>3010</v>
+      </c>
+      <c r="D135" t="s">
+        <v>3020</v>
+      </c>
+      <c r="E135" t="s">
+        <v>3030</v>
+      </c>
+      <c r="F135" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G135" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H135">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="136" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A136">
+        <v>135</v>
+      </c>
+      <c r="B136">
+        <v>14</v>
+      </c>
+      <c r="C136" t="s">
+        <v>3011</v>
+      </c>
+      <c r="D136" t="s">
+        <v>3021</v>
+      </c>
+      <c r="E136" t="s">
+        <v>3031</v>
+      </c>
+      <c r="F136" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G136" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H136">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="137" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A137">
+        <v>136</v>
+      </c>
+      <c r="B137">
+        <v>14</v>
+      </c>
+      <c r="C137" t="s">
+        <v>3012</v>
+      </c>
+      <c r="D137" t="s">
+        <v>3022</v>
+      </c>
+      <c r="E137" t="s">
+        <v>3032</v>
+      </c>
+      <c r="F137" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G137" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H137">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="138" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A138">
+        <v>137</v>
+      </c>
+      <c r="B138">
+        <v>14</v>
+      </c>
+      <c r="C138" t="s">
+        <v>3013</v>
+      </c>
+      <c r="D138" t="s">
+        <v>3023</v>
+      </c>
+      <c r="E138" t="s">
+        <v>3033</v>
+      </c>
+      <c r="F138" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G138" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H138">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="139" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A139">
+        <v>138</v>
+      </c>
+      <c r="B139">
+        <v>14</v>
+      </c>
+      <c r="C139" t="s">
+        <v>3014</v>
+      </c>
+      <c r="D139" t="s">
+        <v>3024</v>
+      </c>
+      <c r="E139" t="s">
+        <v>3034</v>
+      </c>
+      <c r="F139" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G139" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H139">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="140" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A140">
+        <v>139</v>
+      </c>
+      <c r="B140">
+        <v>14</v>
+      </c>
+      <c r="C140" t="s">
+        <v>3015</v>
+      </c>
+      <c r="D140" t="s">
+        <v>3025</v>
+      </c>
+      <c r="E140" t="s">
+        <v>3035</v>
+      </c>
+      <c r="F140" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G140" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H140">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="141" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A141">
+        <v>140</v>
+      </c>
+      <c r="B141">
+        <v>14</v>
+      </c>
+      <c r="C141" t="s">
+        <v>3016</v>
+      </c>
+      <c r="D141" t="s">
+        <v>3026</v>
+      </c>
+      <c r="E141" t="s">
+        <v>3036</v>
+      </c>
+      <c r="F141" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="G141" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="H141">
+        <v>140</v>
       </c>
     </row>
   </sheetData>
@@ -10435,8 +14562,8 @@
       <c r="C2" t="s">
         <v>2931</v>
       </c>
-      <c r="D2">
-        <v>123456</v>
+      <c r="D2" t="s">
+        <v>2976</v>
       </c>
       <c r="E2" t="s">
         <v>2934</v>
@@ -10479,8 +14606,8 @@
       <c r="C3" t="s">
         <v>2932</v>
       </c>
-      <c r="D3">
-        <v>123456</v>
+      <c r="D3" t="s">
+        <v>2976</v>
       </c>
       <c r="E3" t="s">
         <v>2933</v>
@@ -10523,8 +14650,8 @@
       <c r="C4" t="s">
         <v>2930</v>
       </c>
-      <c r="D4">
-        <v>123456</v>
+      <c r="D4" t="s">
+        <v>2976</v>
       </c>
       <c r="E4" t="s">
         <v>2935</v>
@@ -10567,8 +14694,8 @@
       <c r="C5" t="s">
         <v>2937</v>
       </c>
-      <c r="D5">
-        <v>123456</v>
+      <c r="D5" t="s">
+        <v>2976</v>
       </c>
       <c r="E5" t="s">
         <v>2936</v>
@@ -10612,7 +14739,7 @@
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38B320CB-917C-46B8-96F4-A2E982D167ED}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.7109375" bestFit="1" customWidth="1"/>
@@ -10679,7 +14806,27 @@
         <v>2947</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>3037</v>
+      </c>
+      <c r="C4" t="s">
+        <v>3038</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="F4">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -70615,7 +74762,7 @@
         <v>38</v>
       </c>
       <c r="E1" t="s">
-        <v>2978</v>
+        <v>2968</v>
       </c>
       <c r="F1" t="s">
         <v>39</v>
@@ -77590,7 +81737,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>2979</v>
+        <v>2969</v>
       </c>
       <c r="C2" t="s">
         <v>2919</v>
@@ -77619,7 +81766,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>2980</v>
+        <v>2970</v>
       </c>
       <c r="C3" t="s">
         <v>2920</v>
@@ -77670,7 +81817,7 @@
         <v>36</v>
       </c>
       <c r="C1" t="s">
-        <v>2981</v>
+        <v>2971</v>
       </c>
       <c r="D1" t="s">
         <v>32</v>

</xml_diff>

<commit_message>
Fix Reaction Button, Add Score For Table LessonProgress
</commit_message>
<xml_diff>
--- a/src/mocks/greenlight_data.xlsx
+++ b/src/mocks/greenlight_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SmartDrivingLearningSystem\smart_driving_learning_system\src\mocks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09311508-7DE5-4B21-9F11-D23B9CC2813F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{824A3285-B542-411F-83B1-905055CA2C73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="14" activeTab="19" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="14" activeTab="17" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Role" sheetId="1" r:id="rId1"/>
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10949" uniqueCount="3039">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10950" uniqueCount="3039">
   <si>
     <t>id</t>
   </si>
@@ -14335,17 +14335,18 @@
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2F0C51F-F730-40D6-A3D2-B5A208EEA456}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="6.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -14356,52 +14357,61 @@
         <v>43</v>
       </c>
       <c r="D1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C2">
         <v>1</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>2946</v>
+      <c r="D2">
+        <v>90</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>2947</v>
-      </c>
-      <c r="F2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2946</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C3">
         <v>2</v>
       </c>
-      <c r="D3" s="2" t="s">
-        <v>2946</v>
+      <c r="D3">
+        <v>80</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>2947</v>
-      </c>
-      <c r="F3">
+        <v>2946</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="G3">
         <v>1</v>
       </c>
     </row>

</xml_diff>